<commit_message>
BaseTest 失败时挂载页面源码到 Allure；新增 PageSourceUtil
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/search.xlsx
+++ b/src/main/resources/testdata/search.xlsx
@@ -991,7 +991,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" ht="16.85" spans="1:2">
@@ -1007,7 +1007,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>